<commit_message>
feat: update thermal industry types data file with new information
</commit_message>
<xml_diff>
--- a/Data/HeatSpecific/All_info_industry_types_thermal.xlsx
+++ b/Data/HeatSpecific/All_info_industry_types_thermal.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\asher\Desktop\projects\DEUSTO_iDesign_RES\ThermalProfile\data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\asher\Desktop\projects\DEUSTO_iDesign_RES\Data\HeatSpecific\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{95BF68FF-5817-4C39-9F49-781A70CE7858}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4A1A4022-1CE2-40C0-9902-FD6ED31999A4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" activeTab="1" xr2:uid="{612B240B-EA99-41DA-B7DC-32C187B817CA}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{612B240B-EA99-41DA-B7DC-32C187B817CA}"/>
   </bookViews>
   <sheets>
     <sheet name="Thermal" sheetId="5" r:id="rId1"/>
@@ -557,7 +557,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="562" uniqueCount="229">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="562" uniqueCount="227">
   <si>
     <t>Quelle: Fraunhofer ISI 2020 (2018) Erstellung von Anwendungsbilanzen für die Jahre 2018 bis 2020: für die Sektoren Industrie und GHD, Karlsruhe</t>
   </si>
@@ -646,15 +646,6 @@
     <t>%</t>
   </si>
   <si>
-    <t>Fluktuation</t>
-  </si>
-  <si>
-    <t>Base_faktor</t>
-  </si>
-  <si>
-    <t>Peak_faktor</t>
-  </si>
-  <si>
     <t>&gt;1000 °C</t>
   </si>
   <si>
@@ -1244,6 +1235,9 @@
   </si>
   <si>
     <t>Base_factor</t>
+  </si>
+  <si>
+    <t>Fluctuation</t>
   </si>
 </sst>
 </file>
@@ -1789,46 +1783,46 @@
   <sheetData>
     <row r="1" spans="1:18" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
+        <v>34</v>
+      </c>
+      <c r="B1" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="C1" t="s">
+        <v>32</v>
+      </c>
+      <c r="D1" s="7" t="s">
         <v>37</v>
       </c>
-      <c r="B1" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="C1" t="s">
+      <c r="E1" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="F1" s="7" t="s">
+        <v>205</v>
+      </c>
+      <c r="G1" s="7" t="s">
+        <v>203</v>
+      </c>
+      <c r="H1" s="7" t="s">
+        <v>202</v>
+      </c>
+      <c r="I1" s="7" t="s">
+        <v>204</v>
+      </c>
+      <c r="K1" t="s">
+        <v>224</v>
+      </c>
+      <c r="L1" t="s">
+        <v>225</v>
+      </c>
+      <c r="P1" t="s">
+        <v>39</v>
+      </c>
+      <c r="Q1" t="s">
         <v>35</v>
       </c>
-      <c r="D1" s="7" t="s">
+      <c r="R1" t="s">
         <v>40</v>
-      </c>
-      <c r="E1" s="7" t="s">
-        <v>41</v>
-      </c>
-      <c r="F1" s="7" t="s">
-        <v>208</v>
-      </c>
-      <c r="G1" s="7" t="s">
-        <v>206</v>
-      </c>
-      <c r="H1" s="7" t="s">
-        <v>205</v>
-      </c>
-      <c r="I1" s="7" t="s">
-        <v>207</v>
-      </c>
-      <c r="K1" t="s">
-        <v>31</v>
-      </c>
-      <c r="L1" t="s">
-        <v>30</v>
-      </c>
-      <c r="P1" t="s">
-        <v>42</v>
-      </c>
-      <c r="Q1" t="s">
-        <v>38</v>
-      </c>
-      <c r="R1" t="s">
-        <v>43</v>
       </c>
     </row>
     <row r="2" spans="1:18" x14ac:dyDescent="0.3">
@@ -1851,13 +1845,13 @@
         <v>28</v>
       </c>
       <c r="P2" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="Q2" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="R2" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
     </row>
     <row r="3" spans="1:18" x14ac:dyDescent="0.3">
@@ -2509,7 +2503,7 @@
     </row>
     <row r="18" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A18" s="18" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="B18" s="18"/>
       <c r="C18" s="18"/>
@@ -2525,7 +2519,7 @@
     </row>
     <row r="19" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A19" s="18" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="B19" s="18"/>
       <c r="C19" s="18"/>
@@ -2862,75 +2856,75 @@
   <sheetData>
     <row r="1" spans="1:18" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="B1" s="5" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="C1" t="s">
+        <v>32</v>
+      </c>
+      <c r="D1" s="7" t="s">
+        <v>207</v>
+      </c>
+      <c r="E1" s="7" t="s">
+        <v>208</v>
+      </c>
+      <c r="F1" s="7" t="s">
+        <v>209</v>
+      </c>
+      <c r="G1" s="7" t="s">
+        <v>210</v>
+      </c>
+      <c r="H1" s="7" t="s">
+        <v>211</v>
+      </c>
+      <c r="I1" s="7" t="s">
+        <v>212</v>
+      </c>
+      <c r="K1" t="s">
+        <v>224</v>
+      </c>
+      <c r="L1" t="s">
+        <v>225</v>
+      </c>
+      <c r="P1" t="s">
+        <v>39</v>
+      </c>
+      <c r="Q1" t="s">
         <v>35</v>
       </c>
-      <c r="D1" s="7" t="s">
-        <v>210</v>
-      </c>
-      <c r="E1" s="7" t="s">
-        <v>211</v>
-      </c>
-      <c r="F1" s="7" t="s">
-        <v>212</v>
-      </c>
-      <c r="G1" s="7" t="s">
-        <v>213</v>
-      </c>
-      <c r="H1" s="7" t="s">
-        <v>214</v>
-      </c>
-      <c r="I1" s="7" t="s">
-        <v>215</v>
-      </c>
-      <c r="K1" t="s">
-        <v>227</v>
-      </c>
-      <c r="L1" t="s">
-        <v>228</v>
-      </c>
-      <c r="P1" t="s">
-        <v>42</v>
-      </c>
-      <c r="Q1" t="s">
-        <v>38</v>
-      </c>
       <c r="R1" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
     </row>
     <row r="2" spans="1:18" x14ac:dyDescent="0.3">
       <c r="D2" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="E2" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="F2" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="G2" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="H2" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="I2" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="P2" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="Q2" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="R2" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
     </row>
     <row r="3" spans="1:18" x14ac:dyDescent="0.3">
@@ -2941,7 +2935,7 @@
         <v>8</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>216</v>
+        <v>213</v>
       </c>
       <c r="D3" s="3">
         <v>7.0000000000000009</v>
@@ -2982,7 +2976,7 @@
         <v>25</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="D4" s="3">
         <v>10.251046025104602</v>
@@ -3028,7 +3022,7 @@
         <v>23</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>217</v>
+        <v>214</v>
       </c>
       <c r="D5" s="3">
         <v>2.0942408376963351</v>
@@ -3073,7 +3067,7 @@
         <v>21</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="D6" s="3">
         <v>0.99261898701959783</v>
@@ -3119,7 +3113,7 @@
         <v>19</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>218</v>
+        <v>215</v>
       </c>
       <c r="D7" s="3">
         <v>8.9905362776025246</v>
@@ -3164,7 +3158,7 @@
         <v>22</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>219</v>
+        <v>216</v>
       </c>
       <c r="D8" s="3">
         <v>32.58064516129032</v>
@@ -3210,7 +3204,7 @@
         <v>16</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>220</v>
+        <v>217</v>
       </c>
       <c r="D9" s="3">
         <v>3.0349013657056143</v>
@@ -3255,7 +3249,7 @@
         <v>14</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>221</v>
+        <v>218</v>
       </c>
       <c r="D10" s="3">
         <v>1.5615615615615617</v>
@@ -3301,7 +3295,7 @@
         <v>12</v>
       </c>
       <c r="C11" s="4" t="s">
-        <v>222</v>
+        <v>219</v>
       </c>
       <c r="D11" s="3">
         <v>0.38676407391491191</v>
@@ -3342,7 +3336,7 @@
         <v>10</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>223</v>
+        <v>220</v>
       </c>
       <c r="D12" s="3">
         <v>6.3868613138686126</v>
@@ -3388,7 +3382,7 @@
         <v>8</v>
       </c>
       <c r="C13" s="4" t="s">
-        <v>224</v>
+        <v>221</v>
       </c>
       <c r="D13" s="3">
         <v>33.577981651376149</v>
@@ -3434,7 +3428,7 @@
         <v>6</v>
       </c>
       <c r="C14" s="4" t="s">
-        <v>102</v>
+        <v>99</v>
       </c>
       <c r="D14" s="3">
         <v>70.118343195266277</v>
@@ -3480,7 +3474,7 @@
         <v>4</v>
       </c>
       <c r="C15" s="4" t="s">
-        <v>225</v>
+        <v>222</v>
       </c>
       <c r="D15" s="3">
         <v>37.458745874587464</v>
@@ -3526,7 +3520,7 @@
         <v>2</v>
       </c>
       <c r="C16" s="4" t="s">
-        <v>130</v>
+        <v>127</v>
       </c>
       <c r="D16" s="3">
         <v>28.509532062391678</v>
@@ -3582,7 +3576,7 @@
     </row>
     <row r="18" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A18" s="18" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="B18" s="18"/>
       <c r="C18" s="18"/>
@@ -3598,7 +3592,7 @@
     </row>
     <row r="19" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A19" s="18" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="B19" s="18"/>
       <c r="C19" s="18"/>
@@ -3940,40 +3934,40 @@
   <sheetData>
     <row r="1" spans="1:22" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="16" t="s">
+        <v>34</v>
+      </c>
+      <c r="B1" s="17" t="s">
+        <v>33</v>
+      </c>
+      <c r="C1" s="16" t="s">
+        <v>32</v>
+      </c>
+      <c r="E1" s="7" t="s">
         <v>37</v>
       </c>
-      <c r="B1" s="17" t="s">
-        <v>36</v>
-      </c>
-      <c r="C1" s="16" t="s">
+      <c r="F1" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="G1" s="7" t="s">
+        <v>205</v>
+      </c>
+      <c r="H1" s="7" t="s">
+        <v>203</v>
+      </c>
+      <c r="I1" s="7" t="s">
+        <v>202</v>
+      </c>
+      <c r="J1" s="7" t="s">
+        <v>204</v>
+      </c>
+      <c r="M1" t="s">
+        <v>39</v>
+      </c>
+      <c r="N1" t="s">
         <v>35</v>
       </c>
-      <c r="E1" s="7" t="s">
+      <c r="O1" t="s">
         <v>40</v>
-      </c>
-      <c r="F1" s="7" t="s">
-        <v>41</v>
-      </c>
-      <c r="G1" s="7" t="s">
-        <v>208</v>
-      </c>
-      <c r="H1" s="7" t="s">
-        <v>206</v>
-      </c>
-      <c r="I1" s="7" t="s">
-        <v>205</v>
-      </c>
-      <c r="J1" s="7" t="s">
-        <v>207</v>
-      </c>
-      <c r="M1" t="s">
-        <v>42</v>
-      </c>
-      <c r="N1" t="s">
-        <v>38</v>
-      </c>
-      <c r="O1" t="s">
-        <v>43</v>
       </c>
       <c r="R1">
         <v>2018</v>
@@ -3985,12 +3979,12 @@
         <v>2020</v>
       </c>
       <c r="V1" t="s">
-        <v>201</v>
+        <v>198</v>
       </c>
     </row>
     <row r="2" spans="1:22" x14ac:dyDescent="0.3">
       <c r="D2" s="16" t="s">
-        <v>209</v>
+        <v>206</v>
       </c>
       <c r="E2" t="s">
         <v>28</v>
@@ -4011,25 +4005,25 @@
         <v>28</v>
       </c>
       <c r="M2" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="N2" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="O2" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="Q2" t="s">
-        <v>198</v>
+        <v>195</v>
       </c>
       <c r="R2" t="s">
-        <v>196</v>
+        <v>193</v>
       </c>
       <c r="S2" t="s">
-        <v>196</v>
+        <v>193</v>
       </c>
       <c r="T2" t="s">
-        <v>196</v>
+        <v>193</v>
       </c>
     </row>
     <row r="3" spans="1:22" x14ac:dyDescent="0.3">
@@ -4126,7 +4120,7 @@
         <v>22</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>203</v>
+        <v>200</v>
       </c>
       <c r="E5" s="3"/>
       <c r="F5" s="3"/>
@@ -4160,7 +4154,7 @@
         <v>38.111415999999991</v>
       </c>
       <c r="V5" t="s">
-        <v>204</v>
+        <v>201</v>
       </c>
     </row>
     <row r="6" spans="1:22" x14ac:dyDescent="0.3">
@@ -4174,7 +4168,7 @@
         <v>20</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>200</v>
+        <v>197</v>
       </c>
       <c r="E6" s="3"/>
       <c r="F6" s="3"/>
@@ -4209,7 +4203,7 @@
         <v>95.195205999999985</v>
       </c>
       <c r="V6" t="s">
-        <v>202</v>
+        <v>199</v>
       </c>
     </row>
     <row r="7" spans="1:22" x14ac:dyDescent="0.3">
@@ -4347,7 +4341,7 @@
         <v>13</v>
       </c>
       <c r="D10" s="4" t="s">
-        <v>199</v>
+        <v>196</v>
       </c>
       <c r="E10" s="3"/>
       <c r="F10" s="3"/>
@@ -4393,7 +4387,7 @@
         <v>11</v>
       </c>
       <c r="D11" s="4" t="s">
-        <v>197</v>
+        <v>194</v>
       </c>
       <c r="E11" s="3"/>
       <c r="F11" s="3"/>
@@ -4916,7 +4910,7 @@
   <sheetData>
     <row r="1" spans="1:40" x14ac:dyDescent="0.3">
       <c r="A1" s="20" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="B1" s="20"/>
       <c r="C1" s="20"/>
@@ -4930,68 +4924,68 @@
     </row>
     <row r="2" spans="1:40" x14ac:dyDescent="0.3">
       <c r="Q2" t="s">
+        <v>45</v>
+      </c>
+      <c r="R2" t="s">
+        <v>46</v>
+      </c>
+      <c r="S2" t="s">
+        <v>47</v>
+      </c>
+      <c r="T2" t="s">
         <v>48</v>
       </c>
-      <c r="R2" t="s">
+      <c r="U2" t="s">
         <v>49</v>
       </c>
-      <c r="S2" t="s">
+      <c r="V2" t="s">
         <v>50</v>
-      </c>
-      <c r="T2" t="s">
-        <v>51</v>
-      </c>
-      <c r="U2" t="s">
-        <v>52</v>
-      </c>
-      <c r="V2" t="s">
-        <v>53</v>
       </c>
     </row>
     <row r="3" spans="1:40" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="B3" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="C3" t="s">
+        <v>32</v>
+      </c>
+      <c r="D3" t="s">
+        <v>51</v>
+      </c>
+      <c r="F3" t="s">
+        <v>52</v>
+      </c>
+      <c r="G3" t="s">
+        <v>31</v>
+      </c>
+      <c r="H3" t="s">
+        <v>30</v>
+      </c>
+      <c r="I3" t="s">
         <v>36</v>
       </c>
-      <c r="C3" t="s">
-        <v>35</v>
-      </c>
-      <c r="D3" t="s">
-        <v>54</v>
-      </c>
-      <c r="F3" t="s">
-        <v>55</v>
-      </c>
-      <c r="G3" t="s">
-        <v>34</v>
-      </c>
-      <c r="H3" t="s">
-        <v>33</v>
-      </c>
-      <c r="I3" t="s">
+      <c r="J3" t="s">
+        <v>29</v>
+      </c>
+      <c r="L3" t="s">
+        <v>224</v>
+      </c>
+      <c r="M3" t="s">
+        <v>225</v>
+      </c>
+      <c r="O3" t="s">
+        <v>226</v>
+      </c>
+      <c r="Q3" s="20" t="s">
         <v>39</v>
-      </c>
-      <c r="J3" t="s">
-        <v>32</v>
-      </c>
-      <c r="L3" t="s">
-        <v>31</v>
-      </c>
-      <c r="M3" t="s">
-        <v>30</v>
-      </c>
-      <c r="O3" t="s">
-        <v>29</v>
-      </c>
-      <c r="Q3" s="20" t="s">
-        <v>42</v>
       </c>
       <c r="R3" s="20"/>
       <c r="S3" s="20"/>
       <c r="T3" s="20" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="U3" s="20"/>
       <c r="V3" s="20"/>
@@ -5016,57 +5010,57 @@
         <v>27</v>
       </c>
       <c r="Q4" s="20" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="R4" s="20"/>
       <c r="S4" s="20"/>
       <c r="T4" s="20" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="U4" s="20"/>
       <c r="V4" s="20"/>
       <c r="Z4" s="8"/>
       <c r="AA4" s="9" t="s">
+        <v>54</v>
+      </c>
+      <c r="AB4" s="9" t="s">
+        <v>55</v>
+      </c>
+      <c r="AC4" s="9" t="s">
+        <v>56</v>
+      </c>
+      <c r="AD4" s="9" t="s">
         <v>57</v>
       </c>
-      <c r="AB4" s="9" t="s">
+      <c r="AE4" s="9" t="s">
         <v>58</v>
       </c>
-      <c r="AC4" s="9" t="s">
+      <c r="AF4" s="9" t="s">
         <v>59</v>
       </c>
-      <c r="AD4" s="9" t="s">
+      <c r="AG4" s="9" t="s">
         <v>60</v>
       </c>
-      <c r="AE4" s="9" t="s">
+      <c r="AH4" s="9" t="s">
         <v>61</v>
       </c>
-      <c r="AF4" s="9" t="s">
+      <c r="AI4" s="9" t="s">
         <v>62</v>
       </c>
-      <c r="AG4" s="9" t="s">
+      <c r="AJ4" s="9" t="s">
         <v>63</v>
       </c>
-      <c r="AH4" s="9" t="s">
+      <c r="AK4" s="9" t="s">
         <v>64</v>
       </c>
-      <c r="AI4" s="9" t="s">
+      <c r="AL4" s="9" t="s">
         <v>65</v>
       </c>
-      <c r="AJ4" s="9" t="s">
+      <c r="AM4" s="9" t="s">
         <v>66</v>
       </c>
-      <c r="AK4" s="9" t="s">
+      <c r="AN4" s="9" t="s">
         <v>67</v>
-      </c>
-      <c r="AL4" s="9" t="s">
-        <v>68</v>
-      </c>
-      <c r="AM4" s="9" t="s">
-        <v>69</v>
-      </c>
-      <c r="AN4" s="9" t="s">
-        <v>70</v>
       </c>
     </row>
     <row r="5" spans="1:40" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -5080,7 +5074,7 @@
         <v>26</v>
       </c>
       <c r="D5" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
       <c r="F5" s="1">
         <v>4</v>
@@ -5111,7 +5105,7 @@
       </c>
       <c r="S5" s="3"/>
       <c r="Z5" s="10" t="s">
-        <v>72</v>
+        <v>69</v>
       </c>
       <c r="AA5" s="11"/>
       <c r="AB5" s="11"/>
@@ -5122,11 +5116,11 @@
       <c r="AG5" s="11"/>
       <c r="AH5" s="11"/>
       <c r="AI5" s="11" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
       <c r="AJ5" s="11"/>
       <c r="AK5" s="11" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="AL5" s="11"/>
       <c r="AM5" s="11"/>
@@ -5143,7 +5137,7 @@
         <v>24</v>
       </c>
       <c r="D6" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="F6" s="1">
         <v>25</v>
@@ -5179,7 +5173,7 @@
       </c>
       <c r="S6" s="3"/>
       <c r="Z6" s="10" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="AA6" s="11"/>
       <c r="AB6" s="11"/>
@@ -5191,10 +5185,10 @@
       <c r="AH6" s="11"/>
       <c r="AI6" s="11"/>
       <c r="AJ6" s="11" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="AK6" s="11" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="AL6" s="11"/>
       <c r="AM6" s="11"/>
@@ -5211,7 +5205,7 @@
         <v>22</v>
       </c>
       <c r="D7" t="s">
-        <v>79</v>
+        <v>76</v>
       </c>
       <c r="F7" s="1">
         <v>17</v>
@@ -5246,16 +5240,16 @@
       </c>
       <c r="S7" s="3"/>
       <c r="Z7" s="10" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="AA7" s="11"/>
       <c r="AB7" s="11"/>
       <c r="AC7" s="11"/>
       <c r="AD7" s="11" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
       <c r="AE7" s="11" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
       <c r="AF7" s="11"/>
       <c r="AG7" s="11"/>
@@ -5278,7 +5272,7 @@
         <v>20</v>
       </c>
       <c r="D8" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="F8" s="1">
         <v>8</v>
@@ -5322,7 +5316,7 @@
         <v>105</v>
       </c>
       <c r="Z8" s="10" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
       <c r="AA8" s="11"/>
       <c r="AB8" s="11"/>
@@ -5331,10 +5325,10 @@
       <c r="AE8" s="11"/>
       <c r="AF8" s="11"/>
       <c r="AG8" s="11" t="s">
-        <v>85</v>
+        <v>82</v>
       </c>
       <c r="AH8" s="11" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="AI8" s="11"/>
       <c r="AJ8" s="11"/>
@@ -5354,7 +5348,7 @@
         <v>18</v>
       </c>
       <c r="D9" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="F9" s="1">
         <v>8</v>
@@ -5387,10 +5381,10 @@
       <c r="R9" s="6"/>
       <c r="S9" s="3"/>
       <c r="Z9" s="10" t="s">
-        <v>88</v>
+        <v>85</v>
       </c>
       <c r="AA9" s="11" t="s">
-        <v>89</v>
+        <v>86</v>
       </c>
       <c r="AB9" s="11"/>
       <c r="AC9" s="11"/>
@@ -5417,7 +5411,7 @@
         <v>17</v>
       </c>
       <c r="D10" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="F10" s="1">
         <v>16</v>
@@ -5435,7 +5429,7 @@
         <v>35</v>
       </c>
       <c r="K10" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="L10" s="1">
         <v>2.09</v>
@@ -5454,11 +5448,11 @@
       <c r="R10" s="6"/>
       <c r="S10" s="3"/>
       <c r="Z10" s="10" t="s">
-        <v>92</v>
+        <v>89</v>
       </c>
       <c r="AA10" s="11"/>
       <c r="AB10" s="11" t="s">
-        <v>89</v>
+        <v>86</v>
       </c>
       <c r="AC10" s="11"/>
       <c r="AD10" s="11"/>
@@ -5484,7 +5478,7 @@
         <v>15</v>
       </c>
       <c r="D11" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="F11" s="1">
         <v>4</v>
@@ -5502,7 +5496,7 @@
         <v>62</v>
       </c>
       <c r="K11" t="s">
-        <v>94</v>
+        <v>91</v>
       </c>
       <c r="L11" s="1">
         <v>1.39</v>
@@ -5520,7 +5514,7 @@
       <c r="R11" s="6"/>
       <c r="S11" s="3"/>
       <c r="Z11" s="10" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="AA11" s="11"/>
       <c r="AB11" s="11"/>
@@ -5536,7 +5530,7 @@
       <c r="AL11" s="11"/>
       <c r="AM11" s="11"/>
       <c r="AN11" s="11" t="s">
-        <v>89</v>
+        <v>86</v>
       </c>
     </row>
     <row r="12" spans="1:40" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -5550,7 +5544,7 @@
         <v>13</v>
       </c>
       <c r="D12" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
       <c r="F12" s="1">
         <v>4</v>
@@ -5568,7 +5562,7 @@
         <v>62</v>
       </c>
       <c r="K12" t="s">
-        <v>94</v>
+        <v>91</v>
       </c>
       <c r="L12" s="1">
         <v>2.11</v>
@@ -5589,12 +5583,12 @@
       </c>
       <c r="S12" s="3"/>
       <c r="Z12" s="10" t="s">
-        <v>97</v>
+        <v>94</v>
       </c>
       <c r="AA12" s="11"/>
       <c r="AB12" s="11"/>
       <c r="AC12" s="11" t="s">
-        <v>89</v>
+        <v>86</v>
       </c>
       <c r="AD12" s="11"/>
       <c r="AE12" s="11"/>
@@ -5607,7 +5601,7 @@
       <c r="AL12" s="11"/>
       <c r="AM12" s="11"/>
       <c r="AN12" s="11" t="s">
-        <v>98</v>
+        <v>95</v>
       </c>
     </row>
     <row r="13" spans="1:40" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -5621,7 +5615,7 @@
         <v>11</v>
       </c>
       <c r="D13" t="s">
-        <v>99</v>
+        <v>96</v>
       </c>
       <c r="F13" s="1">
         <v>3</v>
@@ -5657,7 +5651,7 @@
         <v>1.4</v>
       </c>
       <c r="Z13" s="10" t="s">
-        <v>100</v>
+        <v>97</v>
       </c>
       <c r="AA13" s="11"/>
       <c r="AB13" s="11"/>
@@ -5672,7 +5666,7 @@
       <c r="AK13" s="11"/>
       <c r="AL13" s="11"/>
       <c r="AM13" s="11" t="s">
-        <v>89</v>
+        <v>86</v>
       </c>
       <c r="AN13" s="11"/>
     </row>
@@ -5687,7 +5681,7 @@
         <v>9</v>
       </c>
       <c r="D14" t="s">
-        <v>101</v>
+        <v>98</v>
       </c>
       <c r="F14" s="1">
         <v>3</v>
@@ -5723,7 +5717,7 @@
       </c>
       <c r="S14" s="3"/>
       <c r="Z14" s="10" t="s">
-        <v>102</v>
+        <v>99</v>
       </c>
       <c r="AA14" s="11"/>
       <c r="AB14" s="11"/>
@@ -5736,14 +5730,14 @@
       <c r="AI14" s="11"/>
       <c r="AJ14" s="11"/>
       <c r="AK14" s="11" t="s">
-        <v>103</v>
+        <v>100</v>
       </c>
       <c r="AL14" s="11" t="s">
-        <v>104</v>
+        <v>101</v>
       </c>
       <c r="AM14" s="11"/>
       <c r="AN14" s="11" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
     </row>
     <row r="15" spans="1:40" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -5757,7 +5751,7 @@
         <v>7</v>
       </c>
       <c r="D15" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="F15" s="1">
         <v>51</v>
@@ -5775,7 +5769,7 @@
         <v>17</v>
       </c>
       <c r="K15" t="s">
-        <v>102</v>
+        <v>99</v>
       </c>
       <c r="L15" s="1">
         <v>2.1800000000000002</v>
@@ -5794,7 +5788,7 @@
       <c r="R15" s="6"/>
       <c r="S15" s="3"/>
       <c r="Z15" s="10" t="s">
-        <v>107</v>
+        <v>104</v>
       </c>
       <c r="AA15" s="11"/>
       <c r="AB15" s="11"/>
@@ -5810,7 +5804,7 @@
       <c r="AL15" s="11"/>
       <c r="AM15" s="11"/>
       <c r="AN15" s="11" t="s">
-        <v>89</v>
+        <v>86</v>
       </c>
     </row>
     <row r="16" spans="1:40" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -5824,7 +5818,7 @@
         <v>5</v>
       </c>
       <c r="D16" t="s">
-        <v>102</v>
+        <v>99</v>
       </c>
       <c r="F16" s="1">
         <v>50</v>
@@ -5842,7 +5836,7 @@
         <v>17</v>
       </c>
       <c r="K16" t="s">
-        <v>102</v>
+        <v>99</v>
       </c>
       <c r="L16" s="1">
         <v>1.34</v>
@@ -5863,7 +5857,7 @@
       </c>
       <c r="S16" s="3"/>
       <c r="Z16" s="10" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="AA16" s="11"/>
       <c r="AB16" s="11"/>
@@ -5879,7 +5873,7 @@
       <c r="AL16" s="11"/>
       <c r="AM16" s="11"/>
       <c r="AN16" s="11" t="s">
-        <v>89</v>
+        <v>86</v>
       </c>
     </row>
     <row r="17" spans="1:40" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -5893,7 +5887,7 @@
         <v>3</v>
       </c>
       <c r="D17" t="s">
-        <v>109</v>
+        <v>106</v>
       </c>
       <c r="F17" s="1">
         <v>52</v>
@@ -5911,7 +5905,7 @@
         <v>16</v>
       </c>
       <c r="K17" t="s">
-        <v>102</v>
+        <v>99</v>
       </c>
       <c r="L17" s="1">
         <v>1.37</v>
@@ -5932,7 +5926,7 @@
       </c>
       <c r="S17" s="3"/>
       <c r="Z17" s="10" t="s">
-        <v>110</v>
+        <v>107</v>
       </c>
       <c r="AA17" s="11"/>
       <c r="AB17" s="11"/>
@@ -5940,23 +5934,23 @@
       <c r="AD17" s="11"/>
       <c r="AE17" s="11"/>
       <c r="AF17" s="11" t="s">
-        <v>111</v>
+        <v>108</v>
       </c>
       <c r="AG17" s="11"/>
       <c r="AH17" s="11" t="s">
-        <v>112</v>
+        <v>109</v>
       </c>
       <c r="AI17" s="11"/>
       <c r="AJ17" s="11" t="s">
-        <v>113</v>
+        <v>110</v>
       </c>
       <c r="AK17" s="11"/>
       <c r="AL17" s="11" t="s">
-        <v>114</v>
+        <v>111</v>
       </c>
       <c r="AM17" s="11"/>
       <c r="AN17" s="11" t="s">
-        <v>115</v>
+        <v>112</v>
       </c>
     </row>
     <row r="18" spans="1:40" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -5970,7 +5964,7 @@
         <v>1</v>
       </c>
       <c r="D18" t="s">
-        <v>116</v>
+        <v>113</v>
       </c>
       <c r="F18" s="1">
         <v>18</v>
@@ -5988,7 +5982,7 @@
         <v>42</v>
       </c>
       <c r="K18" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="L18" s="1"/>
       <c r="M18" s="1"/>
@@ -6036,7 +6030,7 @@
     </row>
     <row r="21" spans="1:40" x14ac:dyDescent="0.3">
       <c r="A21" s="20" t="s">
-        <v>117</v>
+        <v>114</v>
       </c>
       <c r="B21" s="20"/>
       <c r="C21" s="20"/>
@@ -6052,22 +6046,22 @@
     </row>
     <row r="22" spans="1:40" x14ac:dyDescent="0.3">
       <c r="E22" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
       <c r="F22" t="s">
-        <v>119</v>
+        <v>116</v>
       </c>
       <c r="G22" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="H22" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="I22" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="J22" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
     </row>
     <row r="23" spans="1:40" x14ac:dyDescent="0.3">
@@ -6081,7 +6075,7 @@
         <v>26</v>
       </c>
       <c r="D23" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
       <c r="E23" s="12">
         <v>7.3170731707317055E-2</v>
@@ -6120,7 +6114,7 @@
         <v>24</v>
       </c>
       <c r="D24" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="E24" s="12">
         <v>0.10251046025104602</v>
@@ -6159,7 +6153,7 @@
         <v>22</v>
       </c>
       <c r="D25" t="s">
-        <v>79</v>
+        <v>76</v>
       </c>
       <c r="E25" s="12">
         <v>2.0942408376963352E-2</v>
@@ -6201,7 +6195,7 @@
         <v>20</v>
       </c>
       <c r="D26" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="E26" s="12">
         <v>9.926189870195978E-3</v>
@@ -6243,7 +6237,7 @@
         <v>18</v>
       </c>
       <c r="D27" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="E27" s="12">
         <v>8.9905362776025247E-2</v>
@@ -6285,7 +6279,7 @@
         <v>17</v>
       </c>
       <c r="D28" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="E28" s="12">
         <v>0.32580645161290323</v>
@@ -6327,7 +6321,7 @@
         <v>15</v>
       </c>
       <c r="D29" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="E29" s="12">
         <v>3.0349013657056143E-2</v>
@@ -6369,7 +6363,7 @@
         <v>13</v>
       </c>
       <c r="D30" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
       <c r="E30" s="12">
         <v>1.5615615615615617E-2</v>
@@ -6411,7 +6405,7 @@
         <v>11</v>
       </c>
       <c r="D31" t="s">
-        <v>99</v>
+        <v>96</v>
       </c>
       <c r="E31" s="12">
         <v>3.867640739149119E-3</v>
@@ -6453,7 +6447,7 @@
         <v>9</v>
       </c>
       <c r="D32" t="s">
-        <v>101</v>
+        <v>98</v>
       </c>
       <c r="E32" s="12">
         <v>6.3868613138686123E-2</v>
@@ -6495,7 +6489,7 @@
         <v>7</v>
       </c>
       <c r="D33" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="E33" s="12">
         <v>0.33577981651376149</v>
@@ -6537,7 +6531,7 @@
         <v>5</v>
       </c>
       <c r="D34" t="s">
-        <v>102</v>
+        <v>99</v>
       </c>
       <c r="E34" s="12">
         <v>0.70118343195266275</v>
@@ -6579,7 +6573,7 @@
         <v>3</v>
       </c>
       <c r="D35" t="s">
-        <v>109</v>
+        <v>106</v>
       </c>
       <c r="E35" s="12">
         <v>0.37458745874587462</v>
@@ -6621,7 +6615,7 @@
         <v>1</v>
       </c>
       <c r="D36" t="s">
-        <v>116</v>
+        <v>113</v>
       </c>
       <c r="E36" s="12">
         <v>0.28509532062391679</v>
@@ -6682,7 +6676,7 @@
     </row>
     <row r="41" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A41" s="20" t="s">
-        <v>120</v>
+        <v>117</v>
       </c>
       <c r="B41" s="20"/>
       <c r="C41" s="20"/>
@@ -6692,61 +6686,61 @@
       <c r="G41" s="20"/>
       <c r="H41" s="20"/>
       <c r="Q41" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="R41" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="S41" t="s">
-        <v>53</v>
+        <v>50</v>
       </c>
     </row>
     <row r="42" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A42" t="s">
+        <v>34</v>
+      </c>
+      <c r="B42" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="C42" t="s">
+        <v>32</v>
+      </c>
+      <c r="D42" t="s">
+        <v>118</v>
+      </c>
+      <c r="F42" t="s">
         <v>37</v>
       </c>
-      <c r="B42" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="C42" t="s">
-        <v>35</v>
-      </c>
-      <c r="D42" t="s">
-        <v>121</v>
-      </c>
-      <c r="F42" t="s">
-        <v>40</v>
-      </c>
       <c r="G42" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="H42" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
       <c r="I42" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="J42" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="K42" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
       <c r="Q42" s="20" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="R42" s="20"/>
       <c r="S42" s="20"/>
     </row>
     <row r="43" spans="1:19" x14ac:dyDescent="0.3">
       <c r="F43" t="s">
-        <v>123</v>
+        <v>120</v>
       </c>
       <c r="G43" t="s">
-        <v>123</v>
+        <v>120</v>
       </c>
       <c r="H43" t="s">
-        <v>123</v>
+        <v>120</v>
       </c>
       <c r="I43" t="s">
         <v>28</v>
@@ -6758,7 +6752,7 @@
         <v>28</v>
       </c>
       <c r="Q43" s="20" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="R43" s="20"/>
       <c r="S43" s="20"/>
@@ -6774,7 +6768,7 @@
         <v>26</v>
       </c>
       <c r="D44" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
       <c r="F44" s="14">
         <v>0.6</v>
@@ -6818,7 +6812,7 @@
         <v>24</v>
       </c>
       <c r="D45" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="F45" s="14">
         <v>14.7</v>
@@ -6862,7 +6856,7 @@
         <v>22</v>
       </c>
       <c r="D46" t="s">
-        <v>79</v>
+        <v>76</v>
       </c>
       <c r="F46" s="14">
         <v>3.2</v>
@@ -6906,7 +6900,7 @@
         <v>20</v>
       </c>
       <c r="D47" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="F47" s="14">
         <v>3.9</v>
@@ -6950,7 +6944,7 @@
         <v>18</v>
       </c>
       <c r="D48" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="F48" s="14">
         <v>5.7</v>
@@ -6994,7 +6988,7 @@
         <v>17</v>
       </c>
       <c r="D49" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="F49" s="14">
         <v>10.1</v>
@@ -7038,7 +7032,7 @@
         <v>15</v>
       </c>
       <c r="D50" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="F50" s="14">
         <v>2</v>
@@ -7082,7 +7076,7 @@
         <v>13</v>
       </c>
       <c r="D51" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
       <c r="F51" s="14">
         <v>2.6</v>
@@ -7126,7 +7120,7 @@
         <v>11</v>
       </c>
       <c r="D52" t="s">
-        <v>99</v>
+        <v>96</v>
       </c>
       <c r="F52" s="14">
         <v>1.8</v>
@@ -7170,7 +7164,7 @@
         <v>9</v>
       </c>
       <c r="D53" t="s">
-        <v>101</v>
+        <v>98</v>
       </c>
       <c r="F53" s="14">
         <v>3.5</v>
@@ -7214,7 +7208,7 @@
         <v>7</v>
       </c>
       <c r="D54" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="F54" s="14">
         <v>18.3</v>
@@ -7258,7 +7252,7 @@
         <v>5</v>
       </c>
       <c r="D55" t="s">
-        <v>102</v>
+        <v>99</v>
       </c>
       <c r="F55" s="14">
         <v>23.7</v>
@@ -7302,7 +7296,7 @@
         <v>3</v>
       </c>
       <c r="D56" t="s">
-        <v>109</v>
+        <v>106</v>
       </c>
       <c r="F56" s="14">
         <v>22.7</v>
@@ -7346,7 +7340,7 @@
         <v>1</v>
       </c>
       <c r="D57" t="s">
-        <v>116</v>
+        <v>113</v>
       </c>
       <c r="F57" s="14">
         <v>32.9</v>
@@ -7381,7 +7375,7 @@
     </row>
     <row r="59" spans="1:54" x14ac:dyDescent="0.3">
       <c r="A59" s="20" t="s">
-        <v>124</v>
+        <v>121</v>
       </c>
       <c r="B59" s="20"/>
       <c r="C59" s="20"/>
@@ -7391,7 +7385,7 @@
       <c r="G59" s="20"/>
       <c r="H59" s="20"/>
       <c r="M59" s="19" t="s">
-        <v>125</v>
+        <v>122</v>
       </c>
       <c r="N59" s="19"/>
       <c r="O59" s="19"/>
@@ -7399,7 +7393,7 @@
       <c r="Q59" s="19"/>
       <c r="R59" s="19"/>
       <c r="S59" s="21" t="s">
-        <v>126</v>
+        <v>123</v>
       </c>
       <c r="T59" s="22"/>
       <c r="U59" s="22"/>
@@ -7407,7 +7401,7 @@
       <c r="W59" s="22"/>
       <c r="X59" s="22"/>
       <c r="Y59" s="19" t="s">
-        <v>127</v>
+        <v>124</v>
       </c>
       <c r="Z59" s="19"/>
       <c r="AA59" s="19"/>
@@ -7415,7 +7409,7 @@
       <c r="AC59" s="19"/>
       <c r="AD59" s="19"/>
       <c r="AE59" s="19" t="s">
-        <v>128</v>
+        <v>125</v>
       </c>
       <c r="AF59" s="19"/>
       <c r="AG59" s="19"/>
@@ -7423,7 +7417,7 @@
       <c r="AI59" s="19"/>
       <c r="AJ59" s="19"/>
       <c r="AK59" s="19" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="AL59" s="19"/>
       <c r="AM59" s="19"/>
@@ -7431,7 +7425,7 @@
       <c r="AO59" s="19"/>
       <c r="AP59" s="19"/>
       <c r="AQ59" s="19" t="s">
-        <v>129</v>
+        <v>126</v>
       </c>
       <c r="AR59" s="19"/>
       <c r="AS59" s="19"/>
@@ -7439,7 +7433,7 @@
       <c r="AU59" s="19"/>
       <c r="AV59" s="19"/>
       <c r="AW59" s="19" t="s">
-        <v>130</v>
+        <v>127</v>
       </c>
       <c r="AX59" s="19"/>
       <c r="AY59" s="19"/>
@@ -7449,157 +7443,157 @@
     </row>
     <row r="60" spans="1:54" x14ac:dyDescent="0.3">
       <c r="A60" t="s">
+        <v>128</v>
+      </c>
+      <c r="B60" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="C60" t="s">
+        <v>32</v>
+      </c>
+      <c r="D60" t="s">
+        <v>118</v>
+      </c>
+      <c r="F60" t="s">
+        <v>129</v>
+      </c>
+      <c r="G60" t="s">
+        <v>130</v>
+      </c>
+      <c r="H60" t="s">
         <v>131</v>
       </c>
-      <c r="B60" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="C60" t="s">
-        <v>35</v>
-      </c>
-      <c r="D60" t="s">
-        <v>121</v>
-      </c>
-      <c r="F60" t="s">
+      <c r="I60" t="s">
         <v>132</v>
       </c>
-      <c r="G60" t="s">
+      <c r="J60" t="s">
         <v>133</v>
       </c>
-      <c r="H60" t="s">
+      <c r="M60" t="s">
         <v>134</v>
       </c>
-      <c r="I60" t="s">
-        <v>135</v>
-      </c>
-      <c r="J60" t="s">
-        <v>136</v>
-      </c>
-      <c r="M60" t="s">
-        <v>137</v>
-      </c>
       <c r="N60" t="s">
+        <v>129</v>
+      </c>
+      <c r="O60" t="s">
+        <v>130</v>
+      </c>
+      <c r="P60" t="s">
+        <v>131</v>
+      </c>
+      <c r="Q60" t="s">
         <v>132</v>
       </c>
-      <c r="O60" t="s">
+      <c r="R60" t="s">
         <v>133</v>
       </c>
-      <c r="P60" t="s">
+      <c r="S60" t="s">
         <v>134</v>
       </c>
-      <c r="Q60" t="s">
-        <v>135</v>
-      </c>
-      <c r="R60" t="s">
-        <v>136</v>
-      </c>
-      <c r="S60" t="s">
-        <v>137</v>
-      </c>
       <c r="T60" t="s">
+        <v>129</v>
+      </c>
+      <c r="U60" t="s">
+        <v>130</v>
+      </c>
+      <c r="V60" t="s">
+        <v>131</v>
+      </c>
+      <c r="W60" t="s">
         <v>132</v>
       </c>
-      <c r="U60" t="s">
+      <c r="X60" t="s">
         <v>133</v>
       </c>
-      <c r="V60" t="s">
+      <c r="Y60" t="s">
         <v>134</v>
       </c>
-      <c r="W60" t="s">
-        <v>135</v>
-      </c>
-      <c r="X60" t="s">
-        <v>136</v>
-      </c>
-      <c r="Y60" t="s">
-        <v>137</v>
-      </c>
       <c r="Z60" t="s">
+        <v>129</v>
+      </c>
+      <c r="AA60" t="s">
+        <v>130</v>
+      </c>
+      <c r="AB60" t="s">
+        <v>131</v>
+      </c>
+      <c r="AC60" t="s">
         <v>132</v>
       </c>
-      <c r="AA60" t="s">
+      <c r="AD60" t="s">
         <v>133</v>
       </c>
-      <c r="AB60" t="s">
+      <c r="AE60" t="s">
         <v>134</v>
       </c>
-      <c r="AC60" t="s">
-        <v>135</v>
-      </c>
-      <c r="AD60" t="s">
-        <v>136</v>
-      </c>
-      <c r="AE60" t="s">
-        <v>137</v>
-      </c>
       <c r="AF60" t="s">
+        <v>129</v>
+      </c>
+      <c r="AG60" t="s">
+        <v>130</v>
+      </c>
+      <c r="AH60" t="s">
+        <v>131</v>
+      </c>
+      <c r="AI60" t="s">
         <v>132</v>
       </c>
-      <c r="AG60" t="s">
+      <c r="AJ60" t="s">
         <v>133</v>
       </c>
-      <c r="AH60" t="s">
+      <c r="AK60" t="s">
         <v>134</v>
       </c>
-      <c r="AI60" t="s">
-        <v>135</v>
-      </c>
-      <c r="AJ60" t="s">
-        <v>136</v>
-      </c>
-      <c r="AK60" t="s">
-        <v>137</v>
-      </c>
       <c r="AL60" t="s">
+        <v>129</v>
+      </c>
+      <c r="AM60" t="s">
+        <v>130</v>
+      </c>
+      <c r="AN60" t="s">
+        <v>131</v>
+      </c>
+      <c r="AO60" t="s">
         <v>132</v>
       </c>
-      <c r="AM60" t="s">
+      <c r="AP60" t="s">
         <v>133</v>
       </c>
-      <c r="AN60" t="s">
+      <c r="AQ60" t="s">
         <v>134</v>
       </c>
-      <c r="AO60" t="s">
-        <v>135</v>
-      </c>
-      <c r="AP60" t="s">
-        <v>136</v>
-      </c>
-      <c r="AQ60" t="s">
-        <v>137</v>
-      </c>
       <c r="AR60" t="s">
+        <v>129</v>
+      </c>
+      <c r="AS60" t="s">
+        <v>130</v>
+      </c>
+      <c r="AT60" t="s">
+        <v>131</v>
+      </c>
+      <c r="AU60" t="s">
         <v>132</v>
       </c>
-      <c r="AS60" t="s">
+      <c r="AV60" t="s">
         <v>133</v>
       </c>
-      <c r="AT60" t="s">
+      <c r="AW60" t="s">
         <v>134</v>
       </c>
-      <c r="AU60" t="s">
-        <v>135</v>
-      </c>
-      <c r="AV60" t="s">
-        <v>136</v>
-      </c>
-      <c r="AW60" t="s">
-        <v>137</v>
-      </c>
       <c r="AX60" t="s">
+        <v>129</v>
+      </c>
+      <c r="AY60" t="s">
+        <v>130</v>
+      </c>
+      <c r="AZ60" t="s">
+        <v>131</v>
+      </c>
+      <c r="BA60" t="s">
         <v>132</v>
       </c>
-      <c r="AY60" t="s">
+      <c r="BB60" t="s">
         <v>133</v>
-      </c>
-      <c r="AZ60" t="s">
-        <v>134</v>
-      </c>
-      <c r="BA60" t="s">
-        <v>135</v>
-      </c>
-      <c r="BB60" t="s">
-        <v>136</v>
       </c>
     </row>
     <row r="61" spans="1:54" x14ac:dyDescent="0.3">
@@ -7619,7 +7613,7 @@
         <v>28</v>
       </c>
       <c r="M61" t="s">
-        <v>138</v>
+        <v>135</v>
       </c>
       <c r="N61">
         <v>0</v>
@@ -7637,7 +7631,7 @@
         <v>0</v>
       </c>
       <c r="S61" t="s">
-        <v>139</v>
+        <v>136</v>
       </c>
       <c r="T61">
         <v>0</v>
@@ -7655,7 +7649,7 @@
         <v>0</v>
       </c>
       <c r="Y61" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="Z61">
         <v>0.05</v>
@@ -7673,7 +7667,7 @@
         <v>0</v>
       </c>
       <c r="AE61" t="s">
-        <v>141</v>
+        <v>138</v>
       </c>
       <c r="AF61">
         <v>0.02</v>
@@ -7691,7 +7685,7 @@
         <v>0.3</v>
       </c>
       <c r="AK61" t="s">
-        <v>142</v>
+        <v>139</v>
       </c>
       <c r="AL61">
         <v>0</v>
@@ -7709,7 +7703,7 @@
         <v>0</v>
       </c>
       <c r="AQ61" t="s">
-        <v>143</v>
+        <v>140</v>
       </c>
       <c r="AR61">
         <v>0.1</v>
@@ -7727,7 +7721,7 @@
         <v>0</v>
       </c>
       <c r="AW61" t="s">
-        <v>144</v>
+        <v>141</v>
       </c>
       <c r="AX61">
         <v>0.2</v>
@@ -7756,7 +7750,7 @@
         <v>26</v>
       </c>
       <c r="D62" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
       <c r="F62" s="14"/>
       <c r="G62" s="14"/>
@@ -7765,7 +7759,7 @@
       <c r="J62" s="12"/>
       <c r="K62" s="12"/>
       <c r="M62" t="s">
-        <v>145</v>
+        <v>142</v>
       </c>
       <c r="N62">
         <v>0.01</v>
@@ -7783,7 +7777,7 @@
         <v>0.67</v>
       </c>
       <c r="S62" t="s">
-        <v>146</v>
+        <v>143</v>
       </c>
       <c r="T62">
         <v>0.28000000000000003</v>
@@ -7801,7 +7795,7 @@
         <v>0</v>
       </c>
       <c r="Y62" t="s">
-        <v>147</v>
+        <v>144</v>
       </c>
       <c r="Z62">
         <v>0</v>
@@ -7819,7 +7813,7 @@
         <v>0</v>
       </c>
       <c r="AE62" t="s">
-        <v>148</v>
+        <v>145</v>
       </c>
       <c r="AF62">
         <v>0.02</v>
@@ -7837,7 +7831,7 @@
         <v>0.22</v>
       </c>
       <c r="AK62" t="s">
-        <v>149</v>
+        <v>146</v>
       </c>
       <c r="AL62">
         <v>0</v>
@@ -7855,7 +7849,7 @@
         <v>0.33</v>
       </c>
       <c r="AQ62" t="s">
-        <v>150</v>
+        <v>147</v>
       </c>
       <c r="AR62">
         <v>0.9</v>
@@ -7873,7 +7867,7 @@
         <v>0</v>
       </c>
       <c r="AW62" t="s">
-        <v>151</v>
+        <v>148</v>
       </c>
       <c r="AX62">
         <v>0.2</v>
@@ -7902,7 +7896,7 @@
         <v>24</v>
       </c>
       <c r="D63" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="F63" s="13">
         <f>AVERAGE(AR61:AR66)</f>
@@ -7926,7 +7920,7 @@
       </c>
       <c r="K63" s="12"/>
       <c r="M63" t="s">
-        <v>152</v>
+        <v>149</v>
       </c>
       <c r="N63">
         <v>0</v>
@@ -7944,7 +7938,7 @@
         <v>0.8</v>
       </c>
       <c r="S63" t="s">
-        <v>153</v>
+        <v>150</v>
       </c>
       <c r="T63">
         <v>0</v>
@@ -7962,7 +7956,7 @@
         <v>0</v>
       </c>
       <c r="Y63" t="s">
-        <v>154</v>
+        <v>151</v>
       </c>
       <c r="Z63">
         <v>0</v>
@@ -7980,7 +7974,7 @@
         <v>0</v>
       </c>
       <c r="AE63" t="s">
-        <v>155</v>
+        <v>152</v>
       </c>
       <c r="AF63">
         <v>0.02</v>
@@ -7998,7 +7992,7 @@
         <v>0.3</v>
       </c>
       <c r="AK63" t="s">
-        <v>156</v>
+        <v>153</v>
       </c>
       <c r="AL63">
         <v>0</v>
@@ -8016,7 +8010,7 @@
         <v>1</v>
       </c>
       <c r="AQ63" t="s">
-        <v>157</v>
+        <v>154</v>
       </c>
       <c r="AR63">
         <v>0.55000000000000004</v>
@@ -8034,7 +8028,7 @@
         <v>0</v>
       </c>
       <c r="AW63" t="s">
-        <v>158</v>
+        <v>155</v>
       </c>
       <c r="AX63">
         <v>0.2</v>
@@ -8063,7 +8057,7 @@
         <v>22</v>
       </c>
       <c r="D64" t="s">
-        <v>79</v>
+        <v>76</v>
       </c>
       <c r="F64" s="13">
         <f>AVERAGE(Z61:Z63)</f>
@@ -8087,7 +8081,7 @@
       </c>
       <c r="K64" s="12"/>
       <c r="M64" t="s">
-        <v>159</v>
+        <v>156</v>
       </c>
       <c r="N64">
         <v>0</v>
@@ -8105,7 +8099,7 @@
         <v>0.8</v>
       </c>
       <c r="S64" t="s">
-        <v>160</v>
+        <v>157</v>
       </c>
       <c r="T64">
         <v>0</v>
@@ -8123,7 +8117,7 @@
         <v>0</v>
       </c>
       <c r="AE64" t="s">
-        <v>161</v>
+        <v>158</v>
       </c>
       <c r="AF64">
         <v>0.02</v>
@@ -8141,7 +8135,7 @@
         <v>0.32</v>
       </c>
       <c r="AK64" t="s">
-        <v>162</v>
+        <v>159</v>
       </c>
       <c r="AL64">
         <v>0</v>
@@ -8159,7 +8153,7 @@
         <v>1</v>
       </c>
       <c r="AQ64" t="s">
-        <v>163</v>
+        <v>160</v>
       </c>
       <c r="AR64">
         <v>0.4</v>
@@ -8188,7 +8182,7 @@
         <v>20</v>
       </c>
       <c r="D65" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="F65" s="13">
         <f>AVERAGE(AL61:AL74)</f>
@@ -8212,7 +8206,7 @@
       </c>
       <c r="K65" s="12"/>
       <c r="M65" t="s">
-        <v>164</v>
+        <v>161</v>
       </c>
       <c r="N65">
         <v>0</v>
@@ -8230,7 +8224,7 @@
         <v>0.8</v>
       </c>
       <c r="S65" t="s">
-        <v>165</v>
+        <v>162</v>
       </c>
       <c r="T65">
         <v>0</v>
@@ -8248,7 +8242,7 @@
         <v>0</v>
       </c>
       <c r="AE65" t="s">
-        <v>166</v>
+        <v>163</v>
       </c>
       <c r="AF65">
         <v>0.3</v>
@@ -8266,7 +8260,7 @@
         <v>0.65</v>
       </c>
       <c r="AK65" t="s">
-        <v>167</v>
+        <v>164</v>
       </c>
       <c r="AL65">
         <v>0</v>
@@ -8284,7 +8278,7 @@
         <v>0</v>
       </c>
       <c r="AQ65" t="s">
-        <v>168</v>
+        <v>165</v>
       </c>
       <c r="AR65">
         <v>0.2</v>
@@ -8313,7 +8307,7 @@
         <v>18</v>
       </c>
       <c r="D66" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="F66" s="14"/>
       <c r="G66" s="14"/>
@@ -8322,7 +8316,7 @@
       <c r="J66" s="12"/>
       <c r="K66" s="12"/>
       <c r="M66" t="s">
-        <v>169</v>
+        <v>166</v>
       </c>
       <c r="N66">
         <v>0</v>
@@ -8340,7 +8334,7 @@
         <v>0</v>
       </c>
       <c r="S66" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="T66">
         <v>0</v>
@@ -8358,7 +8352,7 @@
         <v>1</v>
       </c>
       <c r="AE66" t="s">
-        <v>171</v>
+        <v>168</v>
       </c>
       <c r="AF66">
         <v>0.3</v>
@@ -8376,7 +8370,7 @@
         <v>0.15</v>
       </c>
       <c r="AK66" t="s">
-        <v>172</v>
+        <v>169</v>
       </c>
       <c r="AL66">
         <v>0</v>
@@ -8394,7 +8388,7 @@
         <v>0</v>
       </c>
       <c r="AQ66" t="s">
-        <v>173</v>
+        <v>170</v>
       </c>
       <c r="AR66">
         <v>1</v>
@@ -8423,7 +8417,7 @@
         <v>17</v>
       </c>
       <c r="D67" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="F67" s="14"/>
       <c r="G67" s="14"/>
@@ -8432,7 +8426,7 @@
       <c r="J67" s="12"/>
       <c r="K67" s="12"/>
       <c r="S67" t="s">
-        <v>174</v>
+        <v>171</v>
       </c>
       <c r="T67">
         <v>0</v>
@@ -8450,7 +8444,7 @@
         <v>0</v>
       </c>
       <c r="AE67" t="s">
-        <v>175</v>
+        <v>172</v>
       </c>
       <c r="AF67">
         <v>7.0000000000000007E-2</v>
@@ -8468,7 +8462,7 @@
         <v>0.56999999999999995</v>
       </c>
       <c r="AK67" t="s">
-        <v>176</v>
+        <v>173</v>
       </c>
       <c r="AL67">
         <v>0</v>
@@ -8497,7 +8491,7 @@
         <v>15</v>
       </c>
       <c r="D68" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="F68" s="14"/>
       <c r="G68" s="14"/>
@@ -8506,7 +8500,7 @@
       <c r="J68" s="12"/>
       <c r="K68" s="12"/>
       <c r="S68" t="s">
-        <v>177</v>
+        <v>174</v>
       </c>
       <c r="T68">
         <v>0</v>
@@ -8524,7 +8518,7 @@
         <v>0</v>
       </c>
       <c r="AE68" t="s">
-        <v>178</v>
+        <v>175</v>
       </c>
       <c r="AF68">
         <v>0</v>
@@ -8542,7 +8536,7 @@
         <v>0.3</v>
       </c>
       <c r="AK68" t="s">
-        <v>179</v>
+        <v>176</v>
       </c>
       <c r="AL68">
         <v>0</v>
@@ -8571,7 +8565,7 @@
         <v>13</v>
       </c>
       <c r="D69" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
       <c r="F69" s="13">
         <f>AVERAGE(AF61:AF76)</f>
@@ -8595,7 +8589,7 @@
       </c>
       <c r="K69" s="12"/>
       <c r="S69" t="s">
-        <v>180</v>
+        <v>177</v>
       </c>
       <c r="T69">
         <v>0</v>
@@ -8613,7 +8607,7 @@
         <v>1</v>
       </c>
       <c r="AE69" t="s">
-        <v>181</v>
+        <v>178</v>
       </c>
       <c r="AF69">
         <v>0</v>
@@ -8631,7 +8625,7 @@
         <v>0.3</v>
       </c>
       <c r="AK69" t="s">
-        <v>182</v>
+        <v>179</v>
       </c>
       <c r="AL69">
         <v>0</v>
@@ -8660,7 +8654,7 @@
         <v>11</v>
       </c>
       <c r="D70" t="s">
-        <v>99</v>
+        <v>96</v>
       </c>
       <c r="F70" s="13">
         <f>AVERAGE(N61:N66)</f>
@@ -8684,7 +8678,7 @@
       </c>
       <c r="K70" s="12"/>
       <c r="S70" t="s">
-        <v>183</v>
+        <v>180</v>
       </c>
       <c r="T70">
         <v>0</v>
@@ -8702,7 +8696,7 @@
         <v>0</v>
       </c>
       <c r="AE70" t="s">
-        <v>184</v>
+        <v>181</v>
       </c>
       <c r="AF70">
         <v>0</v>
@@ -8720,7 +8714,7 @@
         <v>0.3</v>
       </c>
       <c r="AK70" t="s">
-        <v>185</v>
+        <v>182</v>
       </c>
       <c r="AL70">
         <v>0</v>
@@ -8749,7 +8743,7 @@
         <v>9</v>
       </c>
       <c r="D71" t="s">
-        <v>101</v>
+        <v>98</v>
       </c>
       <c r="F71" s="13">
         <f>AVERAGE(T61:T70)</f>
@@ -8773,7 +8767,7 @@
       </c>
       <c r="K71" s="12"/>
       <c r="AE71" t="s">
-        <v>186</v>
+        <v>183</v>
       </c>
       <c r="AF71">
         <v>1</v>
@@ -8791,7 +8785,7 @@
         <v>0</v>
       </c>
       <c r="AK71" t="s">
-        <v>187</v>
+        <v>184</v>
       </c>
       <c r="AL71">
         <v>0</v>
@@ -8820,7 +8814,7 @@
         <v>7</v>
       </c>
       <c r="D72" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="F72" s="14"/>
       <c r="G72" s="14"/>
@@ -8829,7 +8823,7 @@
       <c r="J72" s="12"/>
       <c r="K72" s="12"/>
       <c r="AE72" t="s">
-        <v>188</v>
+        <v>185</v>
       </c>
       <c r="AF72">
         <v>0</v>
@@ -8847,7 +8841,7 @@
         <v>0</v>
       </c>
       <c r="AK72" t="s">
-        <v>189</v>
+        <v>186</v>
       </c>
       <c r="AL72">
         <v>0.3</v>
@@ -8876,7 +8870,7 @@
         <v>5</v>
       </c>
       <c r="D73" t="s">
-        <v>102</v>
+        <v>99</v>
       </c>
       <c r="F73" s="14"/>
       <c r="G73" s="14"/>
@@ -8885,7 +8879,7 @@
       <c r="J73" s="12"/>
       <c r="K73" s="12"/>
       <c r="AE73" t="s">
-        <v>190</v>
+        <v>187</v>
       </c>
       <c r="AF73">
         <v>1</v>
@@ -8903,7 +8897,7 @@
         <v>0</v>
       </c>
       <c r="AK73" t="s">
-        <v>191</v>
+        <v>188</v>
       </c>
       <c r="AL73">
         <v>0</v>
@@ -8932,7 +8926,7 @@
         <v>3</v>
       </c>
       <c r="D74" t="s">
-        <v>109</v>
+        <v>106</v>
       </c>
       <c r="F74" s="14"/>
       <c r="G74" s="14"/>
@@ -8941,7 +8935,7 @@
       <c r="J74" s="12"/>
       <c r="K74" s="12"/>
       <c r="AE74" t="s">
-        <v>192</v>
+        <v>189</v>
       </c>
       <c r="AF74">
         <v>1</v>
@@ -8959,7 +8953,7 @@
         <v>0</v>
       </c>
       <c r="AK74" t="s">
-        <v>193</v>
+        <v>190</v>
       </c>
       <c r="AL74">
         <v>0</v>
@@ -8988,7 +8982,7 @@
         <v>1</v>
       </c>
       <c r="D75" t="s">
-        <v>116</v>
+        <v>113</v>
       </c>
       <c r="F75" s="13">
         <f>AVERAGE(AX61:AX63)</f>
@@ -9012,7 +9006,7 @@
       </c>
       <c r="K75" s="12"/>
       <c r="AE75" t="s">
-        <v>194</v>
+        <v>191</v>
       </c>
       <c r="AF75">
         <v>0.2</v>
@@ -9032,7 +9026,7 @@
     </row>
     <row r="76" spans="1:48" x14ac:dyDescent="0.3">
       <c r="AE76" t="s">
-        <v>195</v>
+        <v>192</v>
       </c>
       <c r="AF76">
         <v>0</v>

</xml_diff>